<commit_message>
chore: update excel reports with patched umlaut urls
</commit_message>
<xml_diff>
--- a/pinyin_CLI_report.xlsx
+++ b/pinyin_CLI_report.xlsx
@@ -5,6 +5,9 @@
   <sheets>
     <sheet name="Pinyin Audio" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pinyin Audio'!$A$1:$J$2001</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -397,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2001"/>
+  <dimension ref="A1:J2001"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,6 +430,9 @@
       <c r="I1" t="str">
         <v>CLI Download Status</v>
       </c>
+      <c r="J1" t="str">
+        <v>__EMPTY</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -26875,6 +26881,9 @@
       <c r="I913" t="str">
         <v>Success</v>
       </c>
+      <c r="J913">
+        <v>1</v>
+      </c>
     </row>
     <row r="914">
       <c r="A914" t="str">
@@ -26904,6 +26913,9 @@
       <c r="I914" t="str">
         <v>Success</v>
       </c>
+      <c r="J914">
+        <v>1</v>
+      </c>
     </row>
     <row r="915">
       <c r="A915" t="str">
@@ -26933,6 +26945,9 @@
       <c r="I915" t="str">
         <v>Success</v>
       </c>
+      <c r="J915">
+        <v>1</v>
+      </c>
     </row>
     <row r="916">
       <c r="A916" t="str">
@@ -26962,6 +26977,9 @@
       <c r="I916" t="str">
         <v>Success</v>
       </c>
+      <c r="J916">
+        <v>1</v>
+      </c>
     </row>
     <row r="917">
       <c r="A917" t="str">
@@ -27444,16 +27462,19 @@
         <v>Success</v>
       </c>
       <c r="F933" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383185/da-phat-am-tieng-trung/audio/lu4.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/lv4.mp3</v>
       </c>
       <c r="G933" t="str">
         <v>Success</v>
       </c>
       <c r="H933" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/lü4.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/lv4.mp3</v>
       </c>
       <c r="I933" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J933">
+        <v>1</v>
       </c>
     </row>
     <row r="934">
@@ -27473,16 +27494,19 @@
         <v>Success</v>
       </c>
       <c r="F934" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383185/da-phat-am-tieng-trung/audio/lu1.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/lv1.mp3</v>
       </c>
       <c r="G934" t="str">
         <v>Success</v>
       </c>
       <c r="H934" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/lü1.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/lv1.mp3</v>
       </c>
       <c r="I934" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J934">
+        <v>1</v>
       </c>
     </row>
     <row r="935">
@@ -27502,16 +27526,19 @@
         <v>Success</v>
       </c>
       <c r="F935" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383186/da-phat-am-tieng-trung/audio/lu2.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/lv2.mp3</v>
       </c>
       <c r="G935" t="str">
         <v>Success</v>
       </c>
       <c r="H935" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/lü2.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/lv2.mp3</v>
       </c>
       <c r="I935" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J935">
+        <v>1</v>
       </c>
     </row>
     <row r="936">
@@ -27531,16 +27558,19 @@
         <v>Success</v>
       </c>
       <c r="F936" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383185/da-phat-am-tieng-trung/audio/lu3.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/lv3.mp3</v>
       </c>
       <c r="G936" t="str">
         <v>Success</v>
       </c>
       <c r="H936" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/lü3.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/lv3.mp3</v>
       </c>
       <c r="I936" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J936">
+        <v>1</v>
       </c>
     </row>
     <row r="937">
@@ -27589,16 +27619,19 @@
         <v>Success</v>
       </c>
       <c r="F938" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383188/da-phat-am-tieng-trung/audio/l%C3%BCe4.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/lve4.mp3</v>
       </c>
       <c r="G938" t="str">
         <v>Success</v>
       </c>
       <c r="H938" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/lüe4.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/lve4.mp3</v>
       </c>
       <c r="I938" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J938">
+        <v>1</v>
       </c>
     </row>
     <row r="939">
@@ -27618,16 +27651,19 @@
         <v>Success</v>
       </c>
       <c r="F939" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383188/da-phat-am-tieng-trung/audio/l%C3%BCe2.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/lve2.mp3</v>
       </c>
       <c r="G939" t="str">
         <v>Success</v>
       </c>
       <c r="H939" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/lüe2.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/lve2.mp3</v>
       </c>
       <c r="I939" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J939">
+        <v>1</v>
       </c>
     </row>
     <row r="940">
@@ -27647,16 +27683,19 @@
         <v>Success</v>
       </c>
       <c r="F940" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383188/da-phat-am-tieng-trung/audio/l%C3%BCe3.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/lve3.mp3</v>
       </c>
       <c r="G940" t="str">
         <v>Success</v>
       </c>
       <c r="H940" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/lüe3.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/lve3.mp3</v>
       </c>
       <c r="I940" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J940">
+        <v>1</v>
       </c>
     </row>
     <row r="941">
@@ -27676,16 +27715,19 @@
         <v>Success</v>
       </c>
       <c r="F941" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383188/da-phat-am-tieng-trung/audio/l%C3%BCe1.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/lve1.mp3</v>
       </c>
       <c r="G941" t="str">
         <v>Success</v>
       </c>
       <c r="H941" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/lüe1.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/lve1.mp3</v>
       </c>
       <c r="I941" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J941">
+        <v>1</v>
       </c>
     </row>
     <row r="942">
@@ -33255,6 +33297,9 @@
       <c r="I1133" t="str">
         <v>Success</v>
       </c>
+      <c r="J1133">
+        <v>1</v>
+      </c>
     </row>
     <row r="1134">
       <c r="A1134" t="str">
@@ -33284,6 +33329,9 @@
       <c r="I1134" t="str">
         <v>Success</v>
       </c>
+      <c r="J1134">
+        <v>1</v>
+      </c>
     </row>
     <row r="1135">
       <c r="A1135" t="str">
@@ -33313,6 +33361,9 @@
       <c r="I1135" t="str">
         <v>Success</v>
       </c>
+      <c r="J1135">
+        <v>1</v>
+      </c>
     </row>
     <row r="1136">
       <c r="A1136" t="str">
@@ -33342,6 +33393,9 @@
       <c r="I1136" t="str">
         <v>Success</v>
       </c>
+      <c r="J1136">
+        <v>1</v>
+      </c>
     </row>
     <row r="1137">
       <c r="A1137" t="str">
@@ -33679,16 +33733,19 @@
         <v>Success</v>
       </c>
       <c r="F1148" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383252/da-phat-am-tieng-trung/audio/nu1.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/nv1.mp3</v>
       </c>
       <c r="G1148" t="str">
         <v>Success</v>
       </c>
       <c r="H1148" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/nü1.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/nv1.mp3</v>
       </c>
       <c r="I1148" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J1148">
+        <v>1</v>
       </c>
     </row>
     <row r="1149">
@@ -33708,16 +33765,19 @@
         <v>Success</v>
       </c>
       <c r="F1149" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383252/da-phat-am-tieng-trung/audio/nu4.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/nv4.mp3</v>
       </c>
       <c r="G1149" t="str">
         <v>Success</v>
       </c>
       <c r="H1149" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/nü4.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/nv4.mp3</v>
       </c>
       <c r="I1149" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J1149">
+        <v>1</v>
       </c>
     </row>
     <row r="1150">
@@ -33737,16 +33797,19 @@
         <v>Success</v>
       </c>
       <c r="F1150" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383252/da-phat-am-tieng-trung/audio/nu2.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/nv2.mp3</v>
       </c>
       <c r="G1150" t="str">
         <v>Success</v>
       </c>
       <c r="H1150" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/nü2.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/nv2.mp3</v>
       </c>
       <c r="I1150" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J1150">
+        <v>1</v>
       </c>
     </row>
     <row r="1151">
@@ -33766,16 +33829,19 @@
         <v>Success</v>
       </c>
       <c r="F1151" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383252/da-phat-am-tieng-trung/audio/nu3.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/nv3.mp3</v>
       </c>
       <c r="G1151" t="str">
         <v>Success</v>
       </c>
       <c r="H1151" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/nü3.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/nv3.mp3</v>
       </c>
       <c r="I1151" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J1151">
+        <v>1</v>
       </c>
     </row>
     <row r="1152">
@@ -33824,16 +33890,19 @@
         <v>Success</v>
       </c>
       <c r="F1153" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383254/da-phat-am-tieng-trung/audio/n%C3%BCe2.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/nve2.mp3</v>
       </c>
       <c r="G1153" t="str">
         <v>Success</v>
       </c>
       <c r="H1153" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/nüe2.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/nve2.mp3</v>
       </c>
       <c r="I1153" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J1153">
+        <v>1</v>
       </c>
     </row>
     <row r="1154">
@@ -33853,16 +33922,19 @@
         <v>Success</v>
       </c>
       <c r="F1154" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383254/da-phat-am-tieng-trung/audio/n%C3%BCe3.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/nve3.mp3</v>
       </c>
       <c r="G1154" t="str">
         <v>Success</v>
       </c>
       <c r="H1154" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/nüe3.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/nve3.mp3</v>
       </c>
       <c r="I1154" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J1154">
+        <v>1</v>
       </c>
     </row>
     <row r="1155">
@@ -33882,16 +33954,19 @@
         <v>Success</v>
       </c>
       <c r="F1155" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383254/da-phat-am-tieng-trung/audio/n%C3%BCe1.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/nve1.mp3</v>
       </c>
       <c r="G1155" t="str">
         <v>Success</v>
       </c>
       <c r="H1155" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/nüe1.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/nve1.mp3</v>
       </c>
       <c r="I1155" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J1155">
+        <v>1</v>
       </c>
     </row>
     <row r="1156">
@@ -33911,16 +33986,19 @@
         <v>Success</v>
       </c>
       <c r="F1156" t="str">
-        <v>https://res.cloudinary.com/zopjocdi/video/upload/v1785383254/da-phat-am-tieng-trung/audio/n%C3%BCe4.mp3</v>
+        <v>https://res.cloudinary.com/zopjocdi/video/upload/da-phat-am-tieng-trung/audio/nve4.mp3</v>
       </c>
       <c r="G1156" t="str">
         <v>Success</v>
       </c>
       <c r="H1156" t="str">
-        <v>https://studycli.org/wp-content/uploads/mp3/nüe4.mp3</v>
+        <v>https://studycli.org/wp-content/uploads/mp3/nve4.mp3</v>
       </c>
       <c r="I1156" t="str">
-        <v>Failed (404)</v>
+        <v>Success</v>
+      </c>
+      <c r="J1156">
+        <v>1</v>
       </c>
     </row>
     <row r="1157">
@@ -58430,7 +58508,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2001"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J2001"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>